<commit_message>
Publish PR preview pr-68
</commit_message>
<xml_diff>
--- a/pr-preview/pr-68/obyvak-skladba-materialu.xlsx
+++ b/pr-preview/pr-68/obyvak-skladba-materialu.xlsx
@@ -736,60 +736,56 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="44" customHeight="1">
-      <c r="A5" s="7" t="n">
+    <row r="5" ht="52" customHeight="1">
+      <c r="A5" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="B5" s="7" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>Akustická deska</t>
         </is>
       </c>
-      <c r="C5" s="7" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>Dřevovláknitá deska ρ 140</t>
         </is>
       </c>
-      <c r="D5" s="8" t="inlineStr">
-        <is>
-          <t>NaturHeld 140, tl. 80 mm (P+D 1880×615)</t>
-        </is>
-      </c>
-      <c r="E5" s="7" t="inlineStr">
-        <is>
-          <t>80 mm</t>
-        </is>
-      </c>
-      <c r="F5" s="9" t="n">
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>NaturHeld 140, 60 mm levá / 100 mm pravá</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>60 / 100 mm</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="n">
         <v>71</v>
       </c>
-      <c r="G5" s="7" t="inlineStr">
+      <c r="G5" s="4" t="inlineStr">
         <is>
           <t>m²</t>
         </is>
       </c>
-      <c r="H5" s="9" t="inlineStr">
+      <c r="H5" s="6" t="inlineStr">
         <is>
           <t>12 %</t>
         </is>
       </c>
-      <c r="I5" s="9" t="n">
+      <c r="I5" s="6" t="n">
         <v>79.52</v>
       </c>
-      <c r="J5" s="10" t="n">
-        <v>534</v>
-      </c>
-      <c r="K5" s="11" t="n">
-        <v>42464</v>
-      </c>
-      <c r="L5" s="7" t="inlineStr">
-        <is>
-          <t>přírodnístavba.cz · https://www.prirodnistavba.cz/drevovlaknita-deska-natur-held-140-kg-m3-1880-615-mm-tl-80-mm-pero-drazka-15725.html</t>
-        </is>
-      </c>
-      <c r="M5" s="7" t="inlineStr">
-        <is>
-          <t>Šroubováno přes GKF do CD @ 625 mm. Bez Flex / bez latí na šikmině.</t>
+      <c r="J5" s="6" t="n"/>
+      <c r="K5" s="6" t="n"/>
+      <c r="L5" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M5" s="4" t="inlineStr">
+        <is>
+          <t>Levá 35.50 m² × 60 mm, pravá 35.50 m² × 100 mm. Šroubováno přes GKF do CD @ 625 mm. Cenu 60 a 100 mm ověřit (80 mm už neplatí).</t>
         </is>
       </c>
     </row>
@@ -1017,7 +1013,7 @@
       </c>
       <c r="M9" s="7" t="inlineStr">
         <is>
-          <t>Kotvení z boku krokve. Modelové svěšení 139 mm, noha 200 mm.</t>
+          <t>Kotvení z boku krokve. Modelové svěšení 73 mm, noha 200 mm.</t>
         </is>
       </c>
     </row>
@@ -1074,7 +1070,7 @@
       </c>
       <c r="M10" s="7" t="inlineStr">
         <is>
-          <t>Pravá šikmina. Nejdelší svěšení v modelu 428 mm (u okapu).</t>
+          <t>Pravá šikmina. Nejdelší svěšení v modelu 322 mm (u okapu).</t>
         </is>
       </c>
     </row>
@@ -1089,12 +1085,12 @@
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>Knauf Unifit 035 160 mm</t>
-        </is>
-      </c>
-      <c r="D11" s="8" t="inlineStr">
-        <is>
-          <t>Knauf Insulation Unifit 035, 160 mm</t>
+          <t>zatím neurčeno</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>zatím neurčeno</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
@@ -1118,15 +1114,11 @@
       <c r="I11" s="9" t="n">
         <v>75.53</v>
       </c>
-      <c r="J11" s="10" t="n">
-        <v>242.24</v>
-      </c>
-      <c r="K11" s="11" t="n">
-        <v>18296</v>
-      </c>
+      <c r="J11" s="9" t="n"/>
+      <c r="K11" s="9" t="n"/>
       <c r="L11" s="7" t="inlineStr">
         <is>
-          <t>DEK Unifit 035 160 mm, 242.24 Kč/m² s DPH, na poptávku · https://www.dek.cz/produkty/detail/1460107750-knauf-unifit-035-160mm-3-84m2-role · TL Unifit 035 · https://www.e-sadrokartony.cz/storage/TL-Knauf-Insulation-Unifit-035.pdf</t>
+          <t>Výrobek zatím neurčen — Petr vybere podle zbylé hloubky.</t>
         </is>
       </c>
       <c r="M11" s="7" t="inlineStr">
@@ -1148,21 +1140,21 @@
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>Knauf Unifit 035 140 mm (L) / plná mezera (P)</t>
-        </is>
-      </c>
-      <c r="D12" s="8" t="inlineStr">
-        <is>
-          <t>Knauf Insulation Unifit 035</t>
+          <t>zatím neurčeno</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>zatím neurčeno</t>
         </is>
       </c>
       <c r="E12" s="7" t="inlineStr">
         <is>
-          <t>L 140 mm / P 429 mm</t>
+          <t>L 74 mm / P 323 mm</t>
         </is>
       </c>
       <c r="F12" s="9" t="n">
-        <v>20.92</v>
+        <v>14.74</v>
       </c>
       <c r="G12" s="7" t="inlineStr">
         <is>
@@ -1175,22 +1167,18 @@
         </is>
       </c>
       <c r="I12" s="9" t="n">
-        <v>23.01</v>
-      </c>
-      <c r="J12" s="10" t="n">
-        <v>1514.29</v>
-      </c>
-      <c r="K12" s="11" t="n">
-        <v>34847</v>
-      </c>
+        <v>16.21</v>
+      </c>
+      <c r="J12" s="9" t="n"/>
+      <c r="K12" s="9" t="n"/>
       <c r="L12" s="7" t="inlineStr">
         <is>
-          <t>DEK Unifit 035 140 mm, 212.00 Kč/m² → 1514.29 Kč/m³ · https://www.dek.cz/produkty/detail/1460107749-knauf-unifit-035-140mm-4-44m2-role · TL Unifit 035 · https://www.e-sadrokartony.cz/storage/TL-Knauf-Insulation-Unifit-035.pdf</t>
+          <t>Výrobek zatím neurčen — Petr vybere podle zbylé hloubky.</t>
         </is>
       </c>
       <c r="M12" s="7" t="inlineStr">
         <is>
-          <t>Levá 140 mm. Pravá plná mezera 429 mm (140+140+150 nebo 200+220), bez vzduchu. Objem z modelu 20.92 m³ (celá vlna šikmin 31.84 − pole 10.92). Specifikace uvádí roli 140 mm 1200×4500; DEK aktuálně 1200×3700 (4,44 m²).</t>
+          <t>Levá 73.7 mm, pravá 323.0 mm nad GKF, pod krokvemi. Objem z modelu 14.74 m³ (celá vlna šikmin 25.65 − pole 10.92).</t>
         </is>
       </c>
     </row>
@@ -1331,7 +1319,7 @@
       <c r="I16" s="15" t="n"/>
       <c r="J16" s="15" t="n"/>
       <c r="K16" s="16" t="n">
-        <v>114673</v>
+        <v>19065</v>
       </c>
       <c r="L16" s="15" t="n"/>
       <c r="M16" s="15" t="n"/>
@@ -1339,7 +1327,7 @@
     <row r="17" ht="36" customHeight="1">
       <c r="A17" s="17" t="inlineStr">
         <is>
-          <t>Neoceněno (chybí v součtu): Povrchová úprava; Podkladní nátěr; Krov (nosná konstrukce)</t>
+          <t>Neoceněno (chybí v součtu): Povrchová úprava; Podkladní nátěr; Akustická deska; Minerální vlna mezi krokve; Minerální vlna plénum; Krov (nosná konstrukce)</t>
         </is>
       </c>
       <c r="B17" s="18" t="n"/>
@@ -1371,8 +1359,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D8" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D9" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D11" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D12" r:id="rId10"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1513,7 +1499,7 @@
         </is>
       </c>
       <c r="F3" s="6" t="n">
-        <v>33.92</v>
+        <v>38.27</v>
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
@@ -1526,7 +1512,7 @@
         </is>
       </c>
       <c r="I3" s="6" t="n">
-        <v>37.31</v>
+        <v>42.1</v>
       </c>
       <c r="J3" s="6" t="n"/>
       <c r="K3" s="6" t="n"/>
@@ -1537,7 +1523,7 @@
       </c>
       <c r="M3" s="4" t="inlineStr">
         <is>
-          <t>11.31 m² × 3,0 = 33.9 kg; s rezervou ≈ 3× 18 kg. Cena na poptávku.</t>
+          <t>12.76 m² × 3,0 = 38.3 kg; s rezervou ≈ 3× 18 kg. Cena na poptávku.</t>
         </is>
       </c>
     </row>
@@ -1566,7 +1552,7 @@
         </is>
       </c>
       <c r="F4" s="6" t="n">
-        <v>28.27</v>
+        <v>31.89</v>
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
@@ -1579,7 +1565,7 @@
         </is>
       </c>
       <c r="I4" s="6" t="n">
-        <v>31.09</v>
+        <v>35.08</v>
       </c>
       <c r="J4" s="6" t="n"/>
       <c r="K4" s="6" t="n"/>
@@ -1590,7 +1576,7 @@
       </c>
       <c r="M4" s="4" t="inlineStr">
         <is>
-          <t>11.31 m² × 2,5 = 28.3 kg; s rezervou ≈ 2× 18 kg. Cena na poptávku.</t>
+          <t>12.76 m² × 2,5 = 31.9 kg; s rezervou ≈ 2× 18 kg. Cena na poptávku.</t>
         </is>
       </c>
     </row>
@@ -1619,7 +1605,7 @@
         </is>
       </c>
       <c r="F5" s="9" t="n">
-        <v>11.31</v>
+        <v>12.76</v>
       </c>
       <c r="G5" s="7" t="inlineStr">
         <is>
@@ -1632,13 +1618,13 @@
         </is>
       </c>
       <c r="I5" s="9" t="n">
-        <v>12.66</v>
+        <v>14.29</v>
       </c>
       <c r="J5" s="10" t="n">
         <v>266</v>
       </c>
       <c r="K5" s="11" t="n">
-        <v>3368</v>
+        <v>3801</v>
       </c>
       <c r="L5" s="7" t="inlineStr">
         <is>
@@ -1676,7 +1662,7 @@
         </is>
       </c>
       <c r="F6" s="6" t="n">
-        <v>1.9</v>
+        <v>1.78</v>
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
@@ -1689,13 +1675,13 @@
         </is>
       </c>
       <c r="I6" s="6" t="n">
-        <v>2.09</v>
+        <v>1.95</v>
       </c>
       <c r="J6" s="6" t="n"/>
       <c r="K6" s="6" t="n"/>
       <c r="L6" s="4" t="inlineStr">
         <is>
-          <t>TL Unifit 035 · https://www.e-sadrokartony.cz/storage/TL-Knauf-Insulation-Unifit-035.pdf</t>
+          <t>Výrobek zatím neurčen — Petr vybere podle zbylé hloubky.</t>
         </is>
       </c>
       <c r="M6" s="4" t="inlineStr">
@@ -1757,7 +1743,7 @@
       </c>
       <c r="M7" s="7" t="inlineStr">
         <is>
-          <t>34 prvků (svislé + spodní). UD 28×27 u zdi 10.46 bm (1 ks). Žádné latě, žádné podložky.</t>
+          <t>34 prvků (svislé + spodní). UD 28×27 u zdi 52.29 bm (5 ks). Žádné latě, žádné podložky.</t>
         </is>
       </c>
     </row>
@@ -1786,7 +1772,7 @@
         </is>
       </c>
       <c r="F8" s="9" t="n">
-        <v>6.76</v>
+        <v>4.98</v>
       </c>
       <c r="G8" s="7" t="inlineStr">
         <is>
@@ -1799,13 +1785,13 @@
         </is>
       </c>
       <c r="I8" s="9" t="n">
-        <v>7.57</v>
+        <v>5.58</v>
       </c>
       <c r="J8" s="10" t="n">
         <v>115.88</v>
       </c>
       <c r="K8" s="11" t="n">
-        <v>877</v>
+        <v>646</v>
       </c>
       <c r="L8" s="7" t="inlineStr">
         <is>
@@ -2014,7 +2000,7 @@
         </is>
       </c>
       <c r="F12" s="6" t="n">
-        <v>31.4</v>
+        <v>10.5</v>
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
@@ -2027,13 +2013,13 @@
         </is>
       </c>
       <c r="I12" s="6" t="n">
-        <v>34.5</v>
+        <v>11.5</v>
       </c>
       <c r="J12" s="12" t="n">
         <v>55</v>
       </c>
       <c r="K12" s="13" t="n">
-        <v>1898</v>
+        <v>633</v>
       </c>
       <c r="L12" s="4" t="inlineStr">
         <is>
@@ -2128,7 +2114,7 @@
         </is>
       </c>
       <c r="F14" s="6" t="n">
-        <v>20.9</v>
+        <v>10.5</v>
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
@@ -2141,13 +2127,13 @@
         </is>
       </c>
       <c r="I14" s="6" t="n">
-        <v>23</v>
+        <v>11.5</v>
       </c>
       <c r="J14" s="12" t="n">
         <v>55</v>
       </c>
       <c r="K14" s="13" t="n">
-        <v>1265</v>
+        <v>633</v>
       </c>
       <c r="L14" s="4" t="inlineStr">
         <is>
@@ -2248,7 +2234,7 @@
       <c r="I17" s="15" t="n"/>
       <c r="J17" s="15" t="n"/>
       <c r="K17" s="16" t="n">
-        <v>16345</v>
+        <v>14648</v>
       </c>
       <c r="L17" s="15" t="n"/>
       <c r="M17" s="15" t="n"/>
@@ -2430,7 +2416,7 @@
         </is>
       </c>
       <c r="F3" s="9" t="n">
-        <v>17.18</v>
+        <v>18.19</v>
       </c>
       <c r="G3" s="7" t="inlineStr">
         <is>
@@ -2443,13 +2429,13 @@
         </is>
       </c>
       <c r="I3" s="9" t="n">
-        <v>19.24</v>
+        <v>20.37</v>
       </c>
       <c r="J3" s="10" t="n">
         <v>96</v>
       </c>
       <c r="K3" s="11" t="n">
-        <v>1847</v>
+        <v>1956</v>
       </c>
       <c r="L3" s="7" t="inlineStr">
         <is>
@@ -2489,7 +2475,7 @@
         </is>
       </c>
       <c r="F4" s="9" t="n">
-        <v>98.40000000000001</v>
+        <v>103.2</v>
       </c>
       <c r="G4" s="7" t="inlineStr">
         <is>
@@ -2502,13 +2488,13 @@
         </is>
       </c>
       <c r="I4" s="9" t="n">
-        <v>108.2</v>
+        <v>113.5</v>
       </c>
       <c r="J4" s="10" t="n">
         <v>29.21</v>
       </c>
       <c r="K4" s="11" t="n">
-        <v>3160</v>
+        <v>3315</v>
       </c>
       <c r="L4" s="7" t="inlineStr">
         <is>
@@ -2548,7 +2534,7 @@
         </is>
       </c>
       <c r="F5" s="9" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G5" s="7" t="inlineStr">
         <is>
@@ -2561,13 +2547,13 @@
         </is>
       </c>
       <c r="I5" s="9" t="n">
-        <v>36.7</v>
+        <v>37.8</v>
       </c>
       <c r="J5" s="10" t="n">
         <v>477</v>
       </c>
       <c r="K5" s="11" t="n">
-        <v>17515</v>
+        <v>18031</v>
       </c>
       <c r="L5" s="7" t="inlineStr">
         <is>
@@ -2658,7 +2644,7 @@
         </is>
       </c>
       <c r="F7" s="6" t="n">
-        <v>1.09</v>
+        <v>1.16</v>
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
@@ -2671,13 +2657,13 @@
         </is>
       </c>
       <c r="I7" s="6" t="n">
-        <v>1.19</v>
+        <v>1.28</v>
       </c>
       <c r="J7" s="6" t="n"/>
       <c r="K7" s="6" t="n"/>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>TL Unifit 035 · https://www.e-sadrokartony.cz/storage/TL-Knauf-Insulation-Unifit-035.pdf</t>
+          <t>Výrobek zatím neurčen — Petr vybere podle zbylé hloubky.</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
@@ -2713,7 +2699,7 @@
         </is>
       </c>
       <c r="F8" s="6" t="n">
-        <v>2.5</v>
+        <v>2.68</v>
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
@@ -2726,13 +2712,13 @@
         </is>
       </c>
       <c r="I8" s="6" t="n">
-        <v>2.75</v>
+        <v>2.94</v>
       </c>
       <c r="J8" s="6" t="n"/>
       <c r="K8" s="6" t="n"/>
       <c r="L8" s="4" t="inlineStr">
         <is>
-          <t>TL Unifit 035 · https://www.e-sadrokartony.cz/storage/TL-Knauf-Insulation-Unifit-035.pdf</t>
+          <t>Výrobek zatím neurčen — Petr vybere podle zbylé hloubky.</t>
         </is>
       </c>
       <c r="M8" s="4" t="inlineStr">
@@ -2772,7 +2758,7 @@
       <c r="I10" s="15" t="n"/>
       <c r="J10" s="15" t="n"/>
       <c r="K10" s="16" t="n">
-        <v>22523</v>
+        <v>23301</v>
       </c>
       <c r="L10" s="15" t="n"/>
       <c r="M10" s="15" t="n"/>
@@ -2821,7 +2807,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M25"/>
+  <dimension ref="A1:M27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2950,7 +2936,7 @@
         </is>
       </c>
       <c r="F3" s="6" t="n">
-        <v>246.92</v>
+        <v>251.28</v>
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
@@ -2963,7 +2949,7 @@
         </is>
       </c>
       <c r="I3" s="6" t="n">
-        <v>271.61</v>
+        <v>276.4</v>
       </c>
       <c r="J3" s="6" t="n"/>
       <c r="K3" s="6" t="n"/>
@@ -2974,7 +2960,7 @@
       </c>
       <c r="M3" s="4" t="inlineStr">
         <is>
-          <t>Šikminy+kastlík 82.31 m² → 246.9 kg; objednat 16× 18 kg. Cena na poptávku Sto.</t>
+          <t>Šikminy+kastlík 83.76 m² → 251.3 kg; objednat 16× 18 kg. Cena na poptávku Sto.</t>
         </is>
       </c>
     </row>
@@ -3003,7 +2989,7 @@
         </is>
       </c>
       <c r="F4" s="6" t="n">
-        <v>205.77</v>
+        <v>209.4</v>
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
@@ -3016,7 +3002,7 @@
         </is>
       </c>
       <c r="I4" s="6" t="n">
-        <v>226.35</v>
+        <v>230.34</v>
       </c>
       <c r="J4" s="6" t="n"/>
       <c r="K4" s="6" t="n"/>
@@ -3027,150 +3013,144 @@
       </c>
       <c r="M4" s="4" t="inlineStr">
         <is>
-          <t>205.8 kg; objednat 13× 18 kg. Cena na poptávku Sto.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="44" customHeight="1">
-      <c r="A5" s="7" t="n">
+          <t>209.4 kg; objednat 13× 18 kg. Cena na poptávku Sto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="52" customHeight="1">
+      <c r="A5" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="B5" s="7" t="inlineStr">
-        <is>
-          <t>NaturHeld 140 — 80 mm</t>
-        </is>
-      </c>
-      <c r="C5" s="7" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>NaturHeld 140 — 60 mm levá</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>Dřevovláknitá deska</t>
         </is>
       </c>
-      <c r="D5" s="8" t="inlineStr">
-        <is>
-          <t>NaturHeld 140 / 80 mm</t>
-        </is>
-      </c>
-      <c r="E5" s="7" t="inlineStr">
-        <is>
-          <t>80 mm</t>
-        </is>
-      </c>
-      <c r="F5" s="9" t="n">
-        <v>71</v>
-      </c>
-      <c r="G5" s="7" t="inlineStr">
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>NaturHeld 140 / 60 mm</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>60 mm</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="n">
+        <v>35.5</v>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
         <is>
           <t>m²</t>
         </is>
       </c>
-      <c r="H5" s="9" t="inlineStr">
+      <c r="H5" s="6" t="inlineStr">
         <is>
           <t>12 %</t>
         </is>
       </c>
-      <c r="I5" s="9" t="n">
-        <v>79.52</v>
-      </c>
-      <c r="J5" s="10" t="n">
-        <v>534</v>
-      </c>
-      <c r="K5" s="11" t="n">
-        <v>42464</v>
-      </c>
-      <c r="L5" s="7" t="inlineStr">
-        <is>
-          <t>přírodnístavba.cz · https://www.prirodnistavba.cz/drevovlaknita-deska-natur-held-140-kg-m3-1880-615-mm-tl-80-mm-pero-drazka-15725.html</t>
-        </is>
-      </c>
-      <c r="M5" s="7" t="inlineStr">
-        <is>
-          <t>Šikminy.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="44" customHeight="1">
-      <c r="A6" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="B6" s="7" t="inlineStr">
-        <is>
-          <t>NaturHeld 140 — 40 mm</t>
-        </is>
-      </c>
-      <c r="C6" s="7" t="inlineStr">
+      <c r="I5" s="6" t="n">
+        <v>39.76</v>
+      </c>
+      <c r="J5" s="6" t="n"/>
+      <c r="K5" s="6" t="n"/>
+      <c r="L5" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M5" s="4" t="inlineStr">
+        <is>
+          <t>Okenní šikmina. Cenu ověřit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="52" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>3b</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>NaturHeld 140 — 100 mm pravá</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
         <is>
           <t>Dřevovláknitá deska</t>
         </is>
       </c>
-      <c r="D6" s="8" t="inlineStr">
-        <is>
-          <t>NaturHeld 140 / 40 mm</t>
-        </is>
-      </c>
-      <c r="E6" s="7" t="inlineStr">
-        <is>
-          <t>40 mm</t>
-        </is>
-      </c>
-      <c r="F6" s="9" t="n">
-        <v>11.31</v>
-      </c>
-      <c r="G6" s="7" t="inlineStr">
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>NaturHeld 140 / 100 mm</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>100 mm</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="n">
+        <v>35.5</v>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
         <is>
           <t>m²</t>
         </is>
       </c>
-      <c r="H6" s="9" t="inlineStr">
+      <c r="H6" s="6" t="inlineStr">
         <is>
           <t>12 %</t>
         </is>
       </c>
-      <c r="I6" s="9" t="n">
-        <v>12.66</v>
-      </c>
-      <c r="J6" s="10" t="n">
-        <v>266</v>
-      </c>
-      <c r="K6" s="11" t="n">
-        <v>3368</v>
-      </c>
-      <c r="L6" s="7" t="inlineStr">
-        <is>
-          <t>přírodnístavba.cz · https://www.prirodnistavba.cz/drevovlaknita-deska-natur-held-140-kg-m3-1250-600-mm-tl-40-mm-15722.html</t>
-        </is>
-      </c>
-      <c r="M6" s="7" t="inlineStr">
-        <is>
-          <t>Kastlík.</t>
+      <c r="I6" s="6" t="n">
+        <v>39.76</v>
+      </c>
+      <c r="J6" s="6" t="n"/>
+      <c r="K6" s="6" t="n"/>
+      <c r="L6" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M6" s="4" t="inlineStr">
+        <is>
+          <t>Šikmina u skříní. Cenu ověřit.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="44" customHeight="1">
       <c r="A7" s="7" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>Parozábrana</t>
+          <t>NaturHeld 140 — 40 mm</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>Jutafol N AL 170 Speciál</t>
+          <t>Dřevovláknitá deska</t>
         </is>
       </c>
       <c r="D7" s="8" t="inlineStr">
         <is>
-          <t>Jutafol N AL 170 Speciál</t>
+          <t>NaturHeld 140 / 40 mm</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>role 75 m²</t>
+          <t>40 mm</t>
         </is>
       </c>
       <c r="F7" s="9" t="n">
-        <v>71</v>
+        <v>12.76</v>
       </c>
       <c r="G7" s="7" t="inlineStr">
         <is>
@@ -3179,55 +3159,55 @@
       </c>
       <c r="H7" s="9" t="inlineStr">
         <is>
-          <t>10 %</t>
+          <t>12 %</t>
         </is>
       </c>
       <c r="I7" s="9" t="n">
-        <v>78.09999999999999</v>
+        <v>14.29</v>
       </c>
       <c r="J7" s="10" t="n">
-        <v>35.73</v>
+        <v>266</v>
       </c>
       <c r="K7" s="11" t="n">
-        <v>2791</v>
+        <v>3801</v>
       </c>
       <c r="L7" s="7" t="inlineStr">
         <is>
-          <t>IZOMAT JUTAFOL N AL 170 Speciál · https://www.izomat.cz/parozabrana-juta-jutafol-n-al-170-special.html · TL https://www.ebau.cz/user/related_files/tl-jutafol-n-170-al-cz.pdf</t>
+          <t>přírodnístavba.cz · https://www.prirodnistavba.cz/drevovlaknita-deska-natur-held-140-kg-m3-1250-600-mm-tl-40-mm-15722.html</t>
         </is>
       </c>
       <c r="M7" s="7" t="inlineStr">
         <is>
-          <t>Šikminy 71.00 m² (+10 % ≈ 78.1 m²). Nad CD, pod vlnou. Spoje JUTAFOL SP AL / SP 1, napojení JUTAFOL MASTIC.</t>
+          <t>Kastlík.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="44" customHeight="1">
       <c r="A8" s="7" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>Sádrokarton RF 12,5</t>
+          <t>Parozábrana</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>GKF/RF</t>
+          <t>Jutafol N AL 170 Speciál</t>
         </is>
       </c>
       <c r="D8" s="8" t="inlineStr">
         <is>
-          <t>Rigips RF 12,5</t>
+          <t>Jutafol N AL 170 Speciál</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>12,5 mm</t>
+          <t>role 75 m²</t>
         </is>
       </c>
       <c r="F8" s="9" t="n">
-        <v>77.76000000000001</v>
+        <v>71</v>
       </c>
       <c r="G8" s="7" t="inlineStr">
         <is>
@@ -3236,46 +3216,46 @@
       </c>
       <c r="H8" s="9" t="inlineStr">
         <is>
-          <t>12 %</t>
+          <t>10 %</t>
         </is>
       </c>
       <c r="I8" s="9" t="n">
-        <v>87.09</v>
+        <v>78.09999999999999</v>
       </c>
       <c r="J8" s="10" t="n">
-        <v>115.88</v>
+        <v>35.73</v>
       </c>
       <c r="K8" s="11" t="n">
-        <v>10092</v>
+        <v>2791</v>
       </c>
       <c r="L8" s="7" t="inlineStr">
         <is>
-          <t>DEK · https://www.dek.cz/produkty/detail/3630042500-sadrokarton-po-deska-rf-12-5mm-1250-2000mm</t>
+          <t>IZOMAT JUTAFOL N AL 170 Speciál · https://www.izomat.cz/parozabrana-juta-jutafol-n-al-170-special.html · TL https://www.ebau.cz/user/related_files/tl-jutafol-n-170-al-cz.pdf</t>
         </is>
       </c>
       <c r="M8" s="7" t="inlineStr">
         <is>
-          <t>Šikminy + víko kastlíku.</t>
+          <t>Šikminy 71.00 m² (+10 % ≈ 78.1 m²). Nad CD, pod vlnou. Spoje JUTAFOL SP AL / SP 1, napojení JUTAFOL MASTIC.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="44" customHeight="1">
       <c r="A9" s="7" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>Sádrokarton GKB/RF 12,5 (basstrapy)</t>
+          <t>Sádrokarton RF 12,5</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>GKB plná</t>
+          <t>GKF/RF</t>
         </is>
       </c>
       <c r="D9" s="8" t="inlineStr">
         <is>
-          <t>Rigips RB/RF 12,5</t>
+          <t>Rigips RF 12,5</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
@@ -3284,7 +3264,7 @@
         </is>
       </c>
       <c r="F9" s="9" t="n">
-        <v>17.18</v>
+        <v>75.98</v>
       </c>
       <c r="G9" s="7" t="inlineStr">
         <is>
@@ -3297,165 +3277,165 @@
         </is>
       </c>
       <c r="I9" s="9" t="n">
-        <v>19.24</v>
+        <v>85.09999999999999</v>
       </c>
       <c r="J9" s="10" t="n">
-        <v>96</v>
+        <v>115.88</v>
       </c>
       <c r="K9" s="11" t="n">
-        <v>1847</v>
+        <v>9861</v>
       </c>
       <c r="L9" s="7" t="inlineStr">
         <is>
-          <t>NonstopStavebniny / DEK RB~GKB orientačně</t>
+          <t>DEK · https://www.dek.cz/produkty/detail/3630042500-sadrokarton-po-deska-rf-12-5mm-1250-2000mm</t>
         </is>
       </c>
       <c r="M9" s="7" t="inlineStr">
         <is>
-          <t>Štíty.</t>
+          <t>Šikminy + víko kastlíku.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="44" customHeight="1">
       <c r="A10" s="7" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>Profil R-CD 60×27</t>
+          <t>Sádrokarton GKB/RF 12,5 (basstrapy)</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>CD profil</t>
+          <t>GKB plná</t>
         </is>
       </c>
       <c r="D10" s="8" t="inlineStr">
         <is>
-          <t>Rigips R-CD</t>
+          <t>Rigips RB/RF 12,5</t>
         </is>
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
-          <t>60×27</t>
+          <t>12,5 mm</t>
         </is>
       </c>
       <c r="F10" s="9" t="n">
-        <v>227.1</v>
+        <v>18.19</v>
       </c>
       <c r="G10" s="7" t="inlineStr">
         <is>
-          <t>bm</t>
+          <t>m²</t>
         </is>
       </c>
       <c r="H10" s="9" t="inlineStr">
         <is>
-          <t>10 %</t>
+          <t>12 %</t>
         </is>
       </c>
       <c r="I10" s="9" t="n">
-        <v>249.8</v>
+        <v>20.37</v>
       </c>
       <c r="J10" s="10" t="n">
-        <v>29.21</v>
+        <v>96</v>
       </c>
       <c r="K10" s="11" t="n">
-        <v>7297</v>
+        <v>1956</v>
       </c>
       <c r="L10" s="7" t="inlineStr">
         <is>
-          <t>DEK R-CD · https://www.dek.cz/produkty/vypis/4167-cd-profily-na-strop/28565-rigips</t>
+          <t>NonstopStavebniny / DEK RB~GKB orientačně</t>
         </is>
       </c>
       <c r="M10" s="7" t="inlineStr">
         <is>
-          <t>Šikminy + kastlík + štíty.</t>
+          <t>Štíty.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="44" customHeight="1">
       <c r="A11" s="7" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>Přímý závěs 200 mm DK Mont</t>
+          <t>Profil R-CD 60×27</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>Přímý závěs 200 mm</t>
+          <t>CD profil</t>
         </is>
       </c>
       <c r="D11" s="8" t="inlineStr">
         <is>
-          <t>DK Mont 3631100170</t>
+          <t>Rigips R-CD</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>200 mm</t>
+          <t>60×27</t>
         </is>
       </c>
       <c r="F11" s="9" t="n">
-        <v>52</v>
+        <v>231.9</v>
       </c>
       <c r="G11" s="7" t="inlineStr">
         <is>
-          <t>ks</t>
+          <t>bm</t>
         </is>
       </c>
       <c r="H11" s="9" t="inlineStr">
         <is>
-          <t>8 %</t>
+          <t>10 %</t>
         </is>
       </c>
       <c r="I11" s="9" t="n">
-        <v>56.2</v>
+        <v>255.1</v>
       </c>
       <c r="J11" s="10" t="n">
-        <v>12.52</v>
+        <v>29.21</v>
       </c>
       <c r="K11" s="11" t="n">
-        <v>703</v>
+        <v>7452</v>
       </c>
       <c r="L11" s="7" t="inlineStr">
         <is>
-          <t>DEK DK Mont 200 mm, balení 100 ks / 1 252,30 Kč s DPH · https://www.dek.cz/produkty/detail/3631100170-primy-zaves-cd-i-drevo-200mm-dkm</t>
+          <t>DEK R-CD · https://www.dek.cz/produkty/vypis/4167-cd-profily-na-strop/28565-rigips</t>
         </is>
       </c>
       <c r="M11" s="7" t="inlineStr">
         <is>
-          <t>Okenní šikmina. Svěšení 139 mm. Balení 100 ks.</t>
+          <t>Šikminy + kastlík + štíty.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="44" customHeight="1">
       <c r="A12" s="7" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>Nonius sada</t>
+          <t>Přímý závěs 200 mm DK Mont</t>
         </is>
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>H+S+2× závlačka</t>
+          <t>Přímý závěs 200 mm</t>
         </is>
       </c>
       <c r="D12" s="8" t="inlineStr">
         <is>
-          <t>Rigips Nonius horní 440 + spodní + 2× závlačka</t>
+          <t>DK Mont 3631100170</t>
         </is>
       </c>
       <c r="E12" s="7" t="inlineStr">
         <is>
-          <t>440</t>
+          <t>200 mm</t>
         </is>
       </c>
       <c r="F12" s="9" t="n">
-        <v>78</v>
+        <v>52</v>
       </c>
       <c r="G12" s="7" t="inlineStr">
         <is>
@@ -3468,51 +3448,51 @@
         </is>
       </c>
       <c r="I12" s="9" t="n">
-        <v>84.2</v>
+        <v>56.2</v>
       </c>
       <c r="J12" s="10" t="n">
-        <v>32.07</v>
+        <v>12.52</v>
       </c>
       <c r="K12" s="11" t="n">
-        <v>2702</v>
+        <v>703</v>
       </c>
       <c r="L12" s="7" t="inlineStr">
         <is>
-          <t>sada: IZOMAT Rigips Nonius horní 440 mm, 1 568,16 Kč/100 ks s DPH · https://www.izomat.cz/zaves-rigips-nonius-horni-340-mm-100-ks-baleni.html; DEK spodní CD · https://www.dek.cz/produkty/detail/3631100745-nonius-spodni-cd-dkm; 2× IZOMAT závlačka · https://www.izomat.cz/pojistna-zavlacka-nonius-dk-mont-100-ks-baleni.html</t>
+          <t>DEK DK Mont 200 mm, balení 100 ks / 1 252,30 Kč s DPH · https://www.dek.cz/produkty/detail/3631100170-primy-zaves-cd-i-drevo-200mm-dkm</t>
         </is>
       </c>
       <c r="M12" s="7" t="inlineStr">
         <is>
-          <t>Pravá šikmina + kastlík. Svěšení šikminy 428 mm, kastlík 406 mm.</t>
+          <t>Okenní šikmina. Svěšení 73 mm. Balení 100 ks.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="44" customHeight="1">
       <c r="A13" s="7" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>Akustický třmen KB517112</t>
+          <t>Nonius sada</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>Třmen + Sylomer</t>
+          <t>H+S+2× závlačka</t>
         </is>
       </c>
       <c r="D13" s="8" t="inlineStr">
         <is>
-          <t>Rigips KB517112</t>
+          <t>Rigips Nonius horní 440 + spodní + 2× závlačka</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>440</t>
         </is>
       </c>
       <c r="F13" s="9" t="n">
-        <v>34</v>
+        <v>78</v>
       </c>
       <c r="G13" s="7" t="inlineStr">
         <is>
@@ -3525,165 +3505,161 @@
         </is>
       </c>
       <c r="I13" s="9" t="n">
-        <v>36.7</v>
+        <v>84.2</v>
       </c>
       <c r="J13" s="10" t="n">
-        <v>477</v>
+        <v>32.07</v>
       </c>
       <c r="K13" s="11" t="n">
-        <v>17515</v>
+        <v>2702</v>
       </c>
       <c r="L13" s="7" t="inlineStr">
         <is>
-          <t>ceník Rigips KB517112 (sci-data / distributor) — ověřit nabídkou</t>
+          <t>sada: IZOMAT Rigips Nonius horní 440 mm, 1 568,16 Kč/100 ks s DPH · https://www.izomat.cz/zaves-rigips-nonius-horni-340-mm-100-ks-baleni.html; DEK spodní CD · https://www.dek.cz/produkty/detail/3631100745-nonius-spodni-cd-dkm; 2× IZOMAT závlačka · https://www.izomat.cz/pojistna-zavlacka-nonius-dk-mont-100-ks-baleni.html</t>
         </is>
       </c>
       <c r="M13" s="7" t="inlineStr">
         <is>
-          <t>Štíty.</t>
+          <t>Pravá šikmina + kastlík. Svěšení šikminy 322 mm, kastlík 406 mm.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="44" customHeight="1">
       <c r="A14" s="7" t="n">
+        <v>11</v>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Akustický třmen KB517112</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>Třmen + Sylomer</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>Rigips KB517112</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F14" s="9" t="n">
+        <v>35</v>
+      </c>
+      <c r="G14" s="7" t="inlineStr">
+        <is>
+          <t>ks</t>
+        </is>
+      </c>
+      <c r="H14" s="9" t="inlineStr">
+        <is>
+          <t>8 %</t>
+        </is>
+      </c>
+      <c r="I14" s="9" t="n">
+        <v>37.8</v>
+      </c>
+      <c r="J14" s="10" t="n">
+        <v>477</v>
+      </c>
+      <c r="K14" s="11" t="n">
+        <v>18031</v>
+      </c>
+      <c r="L14" s="7" t="inlineStr">
+        <is>
+          <t>ceník Rigips KB517112 (sci-data / distributor) — ověřit nabídkou</t>
+        </is>
+      </c>
+      <c r="M14" s="7" t="inlineStr">
+        <is>
+          <t>Štíty.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="52" customHeight="1">
+      <c r="A15" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="B14" s="7" t="inlineStr">
-        <is>
-          <t>Minerální vlna mezi krokve – Knauf Unifit 035 160 mm</t>
-        </is>
-      </c>
-      <c r="C14" s="7" t="inlineStr">
-        <is>
-          <t>Knauf Unifit 035 160 mm</t>
-        </is>
-      </c>
-      <c r="D14" s="8" t="inlineStr">
-        <is>
-          <t>Knauf Insulation Unifit 035 160 mm</t>
-        </is>
-      </c>
-      <c r="E14" s="7" t="inlineStr">
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>Minerální vlna mezi krokve</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>zatím neurčeno</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>zatím neurčeno</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
         <is>
           <t>160 mm</t>
         </is>
       </c>
-      <c r="F14" s="9" t="n">
+      <c r="F15" s="6" t="n">
         <v>68.66</v>
       </c>
-      <c r="G14" s="7" t="inlineStr">
+      <c r="G15" s="4" t="inlineStr">
         <is>
           <t>m²</t>
         </is>
       </c>
-      <c r="H14" s="9" t="inlineStr">
+      <c r="H15" s="6" t="inlineStr">
         <is>
           <t>10 %</t>
         </is>
       </c>
-      <c r="I14" s="9" t="n">
+      <c r="I15" s="6" t="n">
         <v>75.53</v>
       </c>
-      <c r="J14" s="10" t="n">
-        <v>242.24</v>
-      </c>
-      <c r="K14" s="11" t="n">
-        <v>18296</v>
-      </c>
-      <c r="L14" s="7" t="inlineStr">
-        <is>
-          <t>DEK Unifit 035 160 mm, 242.24 Kč/m² s DPH, na poptávku · https://www.dek.cz/produkty/detail/1460107750-knauf-unifit-035-160mm-3-84m2-role · TL Unifit 035 · https://www.e-sadrokartony.cz/storage/TL-Knauf-Insulation-Unifit-035.pdf</t>
-        </is>
-      </c>
-      <c r="M14" s="7" t="inlineStr">
-        <is>
-          <t>m² = sklon 77.52 × (775/875). Řez ~790 mm. Specifikace 1200×4000; DEK 1200×3200.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="44" customHeight="1">
-      <c r="A15" s="7" t="n">
-        <v>13</v>
-      </c>
-      <c r="B15" s="7" t="inlineStr">
-        <is>
-          <t>Minerální vlna plénum – Knauf Unifit 035 140 mm (L) / full gap (R)</t>
-        </is>
-      </c>
-      <c r="C15" s="7" t="inlineStr">
-        <is>
-          <t>Knauf Unifit 035</t>
-        </is>
-      </c>
-      <c r="D15" s="8" t="inlineStr">
-        <is>
-          <t>Knauf Insulation Unifit 035 140 mm</t>
-        </is>
-      </c>
-      <c r="E15" s="7" t="inlineStr">
-        <is>
-          <t>L 140 / P 429 mm</t>
-        </is>
-      </c>
-      <c r="F15" s="9" t="n">
-        <v>20.92</v>
-      </c>
-      <c r="G15" s="7" t="inlineStr">
-        <is>
-          <t>m³</t>
-        </is>
-      </c>
-      <c r="H15" s="9" t="inlineStr">
-        <is>
-          <t>10 %</t>
-        </is>
-      </c>
-      <c r="I15" s="9" t="n">
-        <v>23.01</v>
-      </c>
-      <c r="J15" s="10" t="n">
-        <v>1514.29</v>
-      </c>
-      <c r="K15" s="11" t="n">
-        <v>34847</v>
-      </c>
-      <c r="L15" s="7" t="inlineStr">
-        <is>
-          <t>DEK Unifit 035 140 mm, 212.00 Kč/m² → 1514.29 Kč/m³ · https://www.dek.cz/produkty/detail/1460107749-knauf-unifit-035-140mm-4-44m2-role · TL Unifit 035 · https://www.e-sadrokartony.cz/storage/TL-Knauf-Insulation-Unifit-035.pdf</t>
-        </is>
-      </c>
-      <c r="M15" s="7" t="inlineStr">
-        <is>
-          <t>Levá ×140/80 vůči původním 80 mm, pravá plná mezera 429 mm. Objem modelu 20.92 m³.</t>
+      <c r="J15" s="6" t="n"/>
+      <c r="K15" s="6" t="n"/>
+      <c r="L15" s="4" t="inlineStr">
+        <is>
+          <t>Výrobek zatím neurčen — Petr vybere podle zbylé hloubky.</t>
+        </is>
+      </c>
+      <c r="M15" s="4" t="inlineStr">
+        <is>
+          <t>m² = sklon 77.52 × (775/875). Řez ~790 mm.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="52" customHeight="1">
       <c r="A16" s="4" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Minerální vlna kastlík + štíty</t>
+          <t>Minerální vlna pod krokvemi</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Knauf Unifit 035</t>
-        </is>
-      </c>
-      <c r="D16" s="5" t="inlineStr">
-        <is>
-          <t>Knauf Insulation Unifit 035</t>
+          <t>zatím neurčeno</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>zatím neurčeno</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>kastlík dle modelu · štíty 130.5/300 mm</t>
+          <t>L 74 / P 323 mm</t>
         </is>
       </c>
       <c r="F16" s="6" t="n">
-        <v>5.37</v>
+        <v>14.74</v>
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
@@ -3696,28 +3672,30 @@
         </is>
       </c>
       <c r="I16" s="6" t="n">
-        <v>5.91</v>
+        <v>16.21</v>
       </c>
       <c r="J16" s="6" t="n"/>
       <c r="K16" s="6" t="n"/>
       <c r="L16" s="4" t="inlineStr">
         <is>
-          <t>TL Unifit 035 · https://www.e-sadrokartony.cz/storage/TL-Knauf-Insulation-Unifit-035.pdf</t>
+          <t>Výrobek zatím neurčen — Petr vybere podle zbylé hloubky.</t>
         </is>
       </c>
       <c r="M16" s="4" t="inlineStr">
         <is>
-          <t>Kastlík 1.90 + štíty 3.47 m³. Tloušťky beze změny, stejný výrobek.</t>
+          <t>Nad GKF. Levá 73.7 mm, pravá 323.0 mm. Objem modelu 14.74 m³.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="52" customHeight="1">
-      <c r="A17" s="4" t="n">
-        <v>15</v>
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>13b</t>
+        </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>UD 28×27</t>
+          <t>UD 40° na spoji šikminy</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
@@ -3727,12 +3705,12 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>Rigips UD (obvod kastlíku)</t>
+          <t>UD 28×27 naříznutý a ohnutý na 40°</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>28×27</t>
+          <t>40°</t>
         </is>
       </c>
       <c r="F17" s="6" t="n">
@@ -3751,53 +3729,49 @@
       <c r="I17" s="6" t="n">
         <v>11.5</v>
       </c>
-      <c r="J17" s="12" t="n">
-        <v>29.21</v>
-      </c>
-      <c r="K17" s="13" t="n">
-        <v>336</v>
-      </c>
+      <c r="J17" s="6" t="n"/>
+      <c r="K17" s="6" t="n"/>
       <c r="L17" s="4" t="inlineStr">
         <is>
-          <t>DEK R-CD · https://www.dek.cz/produkty/vypis/4167-cd-profily-na-strop/28565-rigips</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M17" s="4" t="inlineStr">
         <is>
-          <t>U obvodové zdi kastlíku. Cena orientačně jako R-CD — UD ověřit nabídkou.</t>
+          <t>Přišroubovaný z boku CD kastlíku. Šikmé CD se do něj zasunou. Spára akryl + páska 10.46 bm.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="52" customHeight="1">
       <c r="A18" s="4" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Zavětrovací pásky 40×2</t>
+          <t>Minerální vlna kastlík + štíty</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Ocelová páska</t>
+          <t>zatím neurčeno</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>Výrobek dosud nezvolen</t>
+          <t>zatím neurčeno</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>40×2</t>
+          <t>kastlík dle modelu · štíty 130.5/300 mm</t>
         </is>
       </c>
       <c r="F18" s="6" t="n">
-        <v>32.6</v>
+        <v>5.5</v>
       </c>
       <c r="G18" s="4" t="inlineStr">
         <is>
-          <t>bm</t>
+          <t>m³</t>
         </is>
       </c>
       <c r="H18" s="6" t="inlineStr">
@@ -3806,51 +3780,47 @@
         </is>
       </c>
       <c r="I18" s="6" t="n">
-        <v>35.8</v>
-      </c>
-      <c r="J18" s="12" t="n">
-        <v>25</v>
-      </c>
-      <c r="K18" s="13" t="n">
-        <v>896</v>
-      </c>
+        <v>6.05</v>
+      </c>
+      <c r="J18" s="6" t="n"/>
+      <c r="K18" s="6" t="n"/>
       <c r="L18" s="4" t="inlineStr">
         <is>
-          <t>orientační ocelová páska 40×2</t>
+          <t>Výrobek zatím neurčen — Petr vybere podle zbylé hloubky.</t>
         </is>
       </c>
       <c r="M18" s="4" t="inlineStr">
         <is>
-          <t>Nedořešeno: přesný typ.</t>
+          <t>Kastlík 1.78 + štíty 3.72 m³. Tloušťky beze změny, stejný výrobek.</t>
         </is>
       </c>
     </row>
     <row r="19" ht="52" customHeight="1">
       <c r="A19" s="4" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>Spirála Ø160</t>
+          <t>UD 28×27</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>VZT potrubí</t>
+          <t>UD profil</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>Výrobce VZT dosud nezvolen</t>
+          <t>Rigips UD (obvod kastlíku)</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>Ø160</t>
+          <t>28×27</t>
         </is>
       </c>
       <c r="F19" s="6" t="n">
-        <v>31.4</v>
+        <v>52.3</v>
       </c>
       <c r="G19" s="4" t="inlineStr">
         <is>
@@ -3859,59 +3829,59 @@
       </c>
       <c r="H19" s="6" t="inlineStr">
         <is>
-          <t>8 %</t>
+          <t>10 %</t>
         </is>
       </c>
       <c r="I19" s="6" t="n">
-        <v>33.9</v>
+        <v>57.5</v>
       </c>
       <c r="J19" s="12" t="n">
-        <v>180</v>
+        <v>29.21</v>
       </c>
       <c r="K19" s="13" t="n">
-        <v>6099</v>
+        <v>1680</v>
       </c>
       <c r="L19" s="4" t="inlineStr">
         <is>
-          <t>orientační spirála Ø160 pozink</t>
+          <t>DEK R-CD · https://www.dek.cz/produkty/vypis/4167-cd-profily-na-strop/28565-rigips</t>
         </is>
       </c>
       <c r="M19" s="4" t="inlineStr">
         <is>
-          <t>3 trasy v kastlíku.</t>
+          <t>U obvodové zdi kastlíku. Cena orientačně jako R-CD — UD ověřit nabídkou.</t>
         </is>
       </c>
     </row>
     <row r="20" ht="52" customHeight="1">
       <c r="A20" s="4" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>Dropy kastlíku</t>
+          <t>Zavětrovací pásky 40×2</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>Krátký závěs</t>
+          <t>Ocelová páska</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>Dosud nezvolen</t>
+          <t>Výrobek dosud nezvolen</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>20×2</t>
+          <t>40×2</t>
         </is>
       </c>
       <c r="F20" s="6" t="n">
-        <v>17</v>
+        <v>32.6</v>
       </c>
       <c r="G20" s="4" t="inlineStr">
         <is>
-          <t>ks</t>
+          <t>bm</t>
         </is>
       </c>
       <c r="H20" s="6" t="inlineStr">
@@ -3920,51 +3890,51 @@
         </is>
       </c>
       <c r="I20" s="6" t="n">
-        <v>18.7</v>
+        <v>35.8</v>
       </c>
       <c r="J20" s="12" t="n">
-        <v>8</v>
+        <v>25</v>
       </c>
       <c r="K20" s="13" t="n">
-        <v>150</v>
+        <v>896</v>
       </c>
       <c r="L20" s="4" t="inlineStr">
         <is>
-          <t>orientační krátký pásek/drop</t>
+          <t>orientační ocelová páska 40×2</t>
         </is>
       </c>
       <c r="M20" s="4" t="inlineStr">
         <is>
-          <t>Kastlík.</t>
+          <t>Nedořešeno: přesný typ.</t>
         </is>
       </c>
     </row>
     <row r="21" ht="52" customHeight="1">
       <c r="A21" s="4" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>Úhelníky kastlíku (spoj + cleat)</t>
+          <t>Spirála Ø160</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>L-profil</t>
+          <t>VZT potrubí</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>Dosud nezvolen</t>
+          <t>Výrobce VZT dosud nezvolen</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Ø160</t>
         </is>
       </c>
       <c r="F21" s="6" t="n">
-        <v>52.3</v>
+        <v>31.4</v>
       </c>
       <c r="G21" s="4" t="inlineStr">
         <is>
@@ -3973,147 +3943,261 @@
       </c>
       <c r="H21" s="6" t="inlineStr">
         <is>
-          <t>10 %</t>
+          <t>8 %</t>
         </is>
       </c>
       <c r="I21" s="6" t="n">
-        <v>57.5</v>
+        <v>33.9</v>
       </c>
       <c r="J21" s="12" t="n">
-        <v>55</v>
+        <v>180</v>
       </c>
       <c r="K21" s="13" t="n">
-        <v>3164</v>
+        <v>6099</v>
       </c>
       <c r="L21" s="4" t="inlineStr">
         <is>
-          <t>orientační L-profil / tenký úhelník</t>
+          <t>orientační spirála Ø160 pozink</t>
         </is>
       </c>
       <c r="M21" s="4" t="inlineStr">
         <is>
-          <t>Spoj + cleat na pozednici.</t>
+          <t>3 trasy v kastlíku.</t>
         </is>
       </c>
     </row>
     <row r="22" ht="52" customHeight="1">
       <c r="A22" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>Dropy kastlíku</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>Krátký závěs</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>Dosud nezvolen</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>20×2</t>
+        </is>
+      </c>
+      <c r="F22" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="G22" s="4" t="inlineStr">
+        <is>
+          <t>ks</t>
+        </is>
+      </c>
+      <c r="H22" s="6" t="inlineStr">
+        <is>
+          <t>10 %</t>
+        </is>
+      </c>
+      <c r="I22" s="6" t="n">
+        <v>18.7</v>
+      </c>
+      <c r="J22" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="K22" s="13" t="n">
+        <v>150</v>
+      </c>
+      <c r="L22" s="4" t="inlineStr">
+        <is>
+          <t>orientační krátký pásek/drop</t>
+        </is>
+      </c>
+      <c r="M22" s="4" t="inlineStr">
+        <is>
+          <t>Kastlík.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="52" customHeight="1">
+      <c r="A23" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>Úhelníky kastlíku (spoj + cleat)</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>L-profil</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>Dosud nezvolen</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F23" s="6" t="n">
+        <v>20.9</v>
+      </c>
+      <c r="G23" s="4" t="inlineStr">
+        <is>
+          <t>bm</t>
+        </is>
+      </c>
+      <c r="H23" s="6" t="inlineStr">
+        <is>
+          <t>10 %</t>
+        </is>
+      </c>
+      <c r="I23" s="6" t="n">
+        <v>23</v>
+      </c>
+      <c r="J23" s="12" t="n">
+        <v>55</v>
+      </c>
+      <c r="K23" s="13" t="n">
+        <v>1265</v>
+      </c>
+      <c r="L23" s="4" t="inlineStr">
+        <is>
+          <t>orientační L-profil / tenký úhelník</t>
+        </is>
+      </c>
+      <c r="M23" s="4" t="inlineStr">
+        <is>
+          <t>Spoj + cleat na pozednici.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="52" customHeight="1">
+      <c r="A24" s="4" t="n">
         <v>20</v>
       </c>
-      <c r="B22" s="4" t="inlineStr">
+      <c r="B24" s="4" t="inlineStr">
         <is>
           <t>Nástěnné úhelníky kastlíku</t>
         </is>
       </c>
-      <c r="C22" s="4" t="inlineStr">
+      <c r="C24" s="4" t="inlineStr">
         <is>
           <t>Úhelník</t>
         </is>
       </c>
-      <c r="D22" s="4" t="inlineStr">
+      <c r="D24" s="4" t="inlineStr">
         <is>
           <t>Dosud nezvolen</t>
         </is>
       </c>
-      <c r="E22" s="4" t="inlineStr">
+      <c r="E24" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F22" s="6" t="n">
+      <c r="F24" s="6" t="n">
         <v>34</v>
       </c>
-      <c r="G22" s="4" t="inlineStr">
+      <c r="G24" s="4" t="inlineStr">
         <is>
           <t>ks</t>
         </is>
       </c>
-      <c r="H22" s="6" t="inlineStr">
+      <c r="H24" s="6" t="inlineStr">
         <is>
           <t>10 %</t>
         </is>
       </c>
-      <c r="I22" s="6" t="n">
+      <c r="I24" s="6" t="n">
         <v>37.4</v>
       </c>
-      <c r="J22" s="12" t="n">
+      <c r="J24" s="12" t="n">
         <v>35</v>
       </c>
-      <c r="K22" s="13" t="n">
+      <c r="K24" s="13" t="n">
         <v>1309</v>
       </c>
-      <c r="L22" s="4" t="inlineStr">
+      <c r="L24" s="4" t="inlineStr">
         <is>
           <t>orientační nástěnný úhelník</t>
         </is>
       </c>
-      <c r="M22" s="4" t="inlineStr">
+      <c r="M24" s="4" t="inlineStr">
         <is>
           <t>Vzpěra u zdi.</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="22" customHeight="1">
-      <c r="A23" s="2" t="inlineStr"/>
-      <c r="B23" s="3" t="n"/>
-      <c r="C23" s="3" t="n"/>
-      <c r="D23" s="3" t="n"/>
-      <c r="E23" s="3" t="n"/>
-      <c r="F23" s="3" t="n"/>
-      <c r="G23" s="3" t="n"/>
-      <c r="H23" s="3" t="n"/>
-      <c r="I23" s="3" t="n"/>
-      <c r="J23" s="3" t="n"/>
-      <c r="K23" s="3" t="n"/>
-      <c r="L23" s="3" t="n"/>
-      <c r="M23" s="3" t="n"/>
-    </row>
-    <row r="24" ht="24" customHeight="1">
-      <c r="A24" s="14" t="inlineStr">
+    <row r="25" ht="22" customHeight="1">
+      <c r="A25" s="2" t="inlineStr"/>
+      <c r="B25" s="3" t="n"/>
+      <c r="C25" s="3" t="n"/>
+      <c r="D25" s="3" t="n"/>
+      <c r="E25" s="3" t="n"/>
+      <c r="F25" s="3" t="n"/>
+      <c r="G25" s="3" t="n"/>
+      <c r="H25" s="3" t="n"/>
+      <c r="I25" s="3" t="n"/>
+      <c r="J25" s="3" t="n"/>
+      <c r="K25" s="3" t="n"/>
+      <c r="L25" s="3" t="n"/>
+      <c r="M25" s="3" t="n"/>
+    </row>
+    <row r="26" ht="24" customHeight="1">
+      <c r="A26" s="14" t="inlineStr">
         <is>
           <t>SOUČET OCENĚNÝCH POLOŽEK (s rezervou, Kč s DPH)</t>
         </is>
       </c>
-      <c r="B24" s="15" t="n"/>
-      <c r="C24" s="15" t="n"/>
-      <c r="D24" s="15" t="n"/>
-      <c r="E24" s="15" t="n"/>
-      <c r="F24" s="15" t="n"/>
-      <c r="G24" s="15" t="n"/>
-      <c r="H24" s="15" t="n"/>
-      <c r="I24" s="15" t="n"/>
-      <c r="J24" s="15" t="n"/>
-      <c r="K24" s="16" t="n">
-        <v>153876</v>
-      </c>
-      <c r="L24" s="15" t="n"/>
-      <c r="M24" s="15" t="n"/>
-    </row>
-    <row r="25" ht="36" customHeight="1">
-      <c r="A25" s="17" t="inlineStr">
-        <is>
-          <t>Neoceněno (chybí v součtu): StoSilent Top Finish; StoSilent Top Basic; Minerální vlna kastlík + štíty</t>
-        </is>
-      </c>
-      <c r="B25" s="18" t="n"/>
-      <c r="C25" s="18" t="n"/>
-      <c r="D25" s="18" t="n"/>
-      <c r="E25" s="18" t="n"/>
-      <c r="F25" s="18" t="n"/>
-      <c r="G25" s="18" t="n"/>
-      <c r="H25" s="18" t="n"/>
-      <c r="I25" s="18" t="n"/>
-      <c r="J25" s="18" t="n"/>
-      <c r="K25" s="18" t="n"/>
-      <c r="L25" s="18" t="n"/>
-      <c r="M25" s="18" t="n"/>
+      <c r="B26" s="15" t="n"/>
+      <c r="C26" s="15" t="n"/>
+      <c r="D26" s="15" t="n"/>
+      <c r="E26" s="15" t="n"/>
+      <c r="F26" s="15" t="n"/>
+      <c r="G26" s="15" t="n"/>
+      <c r="H26" s="15" t="n"/>
+      <c r="I26" s="15" t="n"/>
+      <c r="J26" s="15" t="n"/>
+      <c r="K26" s="16" t="n">
+        <v>58695</v>
+      </c>
+      <c r="L26" s="15" t="n"/>
+      <c r="M26" s="15" t="n"/>
+    </row>
+    <row r="27" ht="36" customHeight="1">
+      <c r="A27" s="17" t="inlineStr">
+        <is>
+          <t>Neoceněno (chybí v součtu): StoSilent Top Finish; StoSilent Top Basic; NaturHeld 140 — 60 mm levá; NaturHeld 140 — 100 mm pravá; Minerální vlna mezi krokve; Minerální vlna pod krokvemi; UD 40° na spoji šikminy; Minerální vlna kastlík + štíty</t>
+        </is>
+      </c>
+      <c r="B27" s="18" t="n"/>
+      <c r="C27" s="18" t="n"/>
+      <c r="D27" s="18" t="n"/>
+      <c r="E27" s="18" t="n"/>
+      <c r="F27" s="18" t="n"/>
+      <c r="G27" s="18" t="n"/>
+      <c r="H27" s="18" t="n"/>
+      <c r="I27" s="18" t="n"/>
+      <c r="J27" s="18" t="n"/>
+      <c r="K27" s="18" t="n"/>
+      <c r="L27" s="18" t="n"/>
+      <c r="M27" s="18" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A25:M25"/>
+    <mergeCell ref="A27:M27"/>
     <mergeCell ref="A2:M2"/>
-    <mergeCell ref="A24:J24"/>
-    <mergeCell ref="A23:M23"/>
+    <mergeCell ref="A26:J26"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId1"/>
@@ -4128,8 +4212,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D12" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D13" r:id="rId11"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D14" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D15" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D16" r:id="rId14"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4288,7 +4370,7 @@
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>11.31 m²</t>
+          <t>12.76 m²</t>
         </is>
       </c>
     </row>
@@ -4300,7 +4382,7 @@
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>8.32 m²</t>
+          <t>8.92 m²</t>
         </is>
       </c>
     </row>

</xml_diff>